<commit_message>
feat(J01): ajout des feuilles de cas pratiques dans le classeur
</commit_message>
<xml_diff>
--- a/01-Fondamentaux/J01-References-cellules/exercices/Classeur-J01.xlsx
+++ b/01-Fondamentaux/J01-References-cellules/exercices/Classeur-J01.xlsx
@@ -5,21 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\excel-data-bootcamp\Jour1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\excel-data-bootcamp\01-Fondamentaux\J01-References-cellules\exercices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B441D56C-38A6-4C4D-B2B9-BAD191465313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1F3F02-E5FD-4BD1-984A-8FA4F369A8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F0BD2965-0CC7-4BBC-A95B-06709D4805A6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="6" xr2:uid="{F0BD2965-0CC7-4BBC-A95B-06709D4805A6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
-    <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
-    <sheet name="Feuil4" sheetId="4" r:id="rId4"/>
-    <sheet name="Feuil5" sheetId="5" r:id="rId5"/>
-    <sheet name="Feuil8" sheetId="9" r:id="rId6"/>
-    <sheet name="Feuil7" sheetId="8" r:id="rId7"/>
+    <sheet name="Cas 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Cas 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Cas 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Cas 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Cas 5" sheetId="5" r:id="rId5"/>
+    <sheet name="Cas 8" sheetId="9" r:id="rId6"/>
+    <sheet name="Cas 7" sheetId="10" r:id="rId7"/>
+    <sheet name="Cas 6" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1073,6 +1074,22 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E429AA9-4CF0-4F7D-ADFC-6D0204079ED7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f ca="1">A1</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7006AE07-9D5E-444D-AA5A-667E73B307B2}">
   <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>